<commit_message>
Update payments and imports
</commit_message>
<xml_diff>
--- a/docs/import-template-v2.xlsx
+++ b/docs/import-template-v2.xlsx
@@ -4,17 +4,18 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
-    <sheet name="suppliers" sheetId="2" r:id="rId2"/>
-    <sheet name="employees" sheetId="3" r:id="rId3"/>
-    <sheet name="categories" sheetId="4" r:id="rId4"/>
-    <sheet name="ingredients" sheetId="5" r:id="rId5"/>
-    <sheet name="products" sheetId="6" r:id="rId6"/>
-    <sheet name="product_ingredients" sheetId="7" r:id="rId7"/>
-    <sheet name="product_additional_ingredients" sheetId="8" r:id="rId8"/>
-    <sheet name="restaurant_tables" sheetId="9" r:id="rId9"/>
-    <sheet name="discounts" sheetId="10" r:id="rId10"/>
-    <sheet name="surcharges" sheetId="11" r:id="rId11"/>
-    <sheet name="receipt_preferences" sheetId="12" r:id="rId12"/>
+    <sheet name="payment_methods" sheetId="2" r:id="rId2"/>
+    <sheet name="suppliers" sheetId="3" r:id="rId3"/>
+    <sheet name="employees" sheetId="4" r:id="rId4"/>
+    <sheet name="categories" sheetId="5" r:id="rId5"/>
+    <sheet name="ingredients" sheetId="6" r:id="rId6"/>
+    <sheet name="products" sheetId="7" r:id="rId7"/>
+    <sheet name="product_ingredients" sheetId="8" r:id="rId8"/>
+    <sheet name="product_additional_ingredients" sheetId="9" r:id="rId9"/>
+    <sheet name="restaurant_tables" sheetId="10" r:id="rId10"/>
+    <sheet name="discounts" sheetId="11" r:id="rId11"/>
+    <sheet name="surcharges" sheetId="12" r:id="rId12"/>
+    <sheet name="receipt_preferences" sheetId="13" r:id="rId13"/>
   </sheets>
 </workbook>
 </file>
@@ -531,6 +532,41 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B3"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>name</v>
+      </c>
+      <c r="B1" t="str">
+        <v>tableType</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Mesa 1</v>
+      </c>
+      <c r="B2" t="str">
+        <v>dine-in</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Takeaway</v>
+      </c>
+      <c r="B3" t="str">
+        <v>to-go</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:B3"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H2"/>
   <sheetData>
     <row r="1">
@@ -592,7 +628,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B3"/>
   <sheetData>
@@ -627,7 +663,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H2"/>
   <sheetData>
@@ -692,6 +728,49 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B4"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>name</v>
+      </c>
+      <c r="B1" t="str">
+        <v>isActive</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Efectivo</v>
+      </c>
+      <c r="B2" t="str">
+        <v>true</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Tarjeta</v>
+      </c>
+      <c r="B3" t="str">
+        <v>true</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Transferencia</v>
+      </c>
+      <c r="B4" t="str">
+        <v>true</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:B4"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C2"/>
   <sheetData>
     <row r="1">
@@ -723,7 +802,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C2"/>
   <sheetData>
@@ -756,7 +835,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:A2"/>
   <sheetData>
@@ -777,7 +856,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E2"/>
   <sheetData>
@@ -822,7 +901,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E2"/>
   <sheetData>
@@ -867,7 +946,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C2"/>
   <sheetData>
@@ -900,7 +979,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D2"/>
   <sheetData>
@@ -937,39 +1016,4 @@
     <ignoredError numberStoredAsText="1" sqref="A1:D2"/>
   </ignoredErrors>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B3"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>name</v>
-      </c>
-      <c r="B1" t="str">
-        <v>tableType</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Mesa 1</v>
-      </c>
-      <c r="B2" t="str">
-        <v>dine-in</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Takeaway</v>
-      </c>
-      <c r="B3" t="str">
-        <v>to-go</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B3"/>
-  </ignoredErrors>
-</worksheet>
 </file>
</xml_diff>